<commit_message>
feat: Hoan thien he thong, ho tro da thue suat (5%, 8%, 10%), clean code va fix triet de 8 loi tiem an
</commit_message>
<xml_diff>
--- a/templates/ĐĐH Mẫu.xlsx
+++ b/templates/ĐĐH Mẫu.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="50">
   <si>
     <t xml:space="preserve">                CÔNG TY CP VIỆT NAM GRAPHENE GLOBAL</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>Số: {so_don_dat_hang}</t>
-  </si>
-  <si>
-    <t>Kính gửi: Quý {ten_cong_ty}</t>
   </si>
   <si>
     <r>
@@ -114,6 +111,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
       <t>-</t>
     </r>
     <r>
@@ -644,7 +647,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="13"/>
+      <sz val="7"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
@@ -655,14 +659,13 @@
       <charset val="2"/>
     </font>
     <font>
-      <sz val="7"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="13"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
@@ -1827,22 +1830,20 @@
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
     </row>
-    <row r="10" ht="27" customHeight="1" spans="1:6">
-      <c r="A10" s="11" t="s">
-        <v>7</v>
-      </c>
+    <row r="10" ht="16" customHeight="1" spans="1:6">
+      <c r="A10" s="11"/>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
       <c r="F10" s="11"/>
     </row>
-    <row r="11" ht="16.8" hidden="1" spans="1:6">
+    <row r="11" ht="16.8" spans="1:6">
       <c r="A11" s="12"/>
     </row>
     <row r="12" ht="16.8" spans="1:6">
       <c r="A12" s="42" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
@@ -1850,9 +1851,9 @@
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
     </row>
-    <row r="13" ht="16.8" hidden="1" spans="1:6">
+    <row r="13" ht="16.8" spans="1:6">
       <c r="A13" s="42" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
@@ -1860,9 +1861,9 @@
       <c r="E13" s="14"/>
       <c r="F13" s="14"/>
     </row>
-    <row r="14" ht="35.25" customHeight="1" spans="1:6">
+    <row r="14" ht="22" customHeight="1" spans="1:6">
       <c r="A14" s="43" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
@@ -1880,83 +1881,83 @@
     </row>
     <row r="16" ht="16.8" spans="1:6">
       <c r="A16" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="C16" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="D16" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="E16" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="F16" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="18" t="s">
+    </row>
+    <row r="17" ht="33" customHeight="1" spans="1:8">
+      <c r="A17" s="19" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" ht="33.6" spans="1:8">
-      <c r="A17" s="19" t="s">
+      <c r="B17" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="C17" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="D17" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="E17" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="22" t="s">
+      <c r="F17" s="23" t="s">
         <v>21</v>
-      </c>
-      <c r="F17" s="23" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="18" ht="16.8" spans="1:8">
       <c r="A18" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
       <c r="D18" s="17"/>
       <c r="E18" s="17"/>
       <c r="F18" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" ht="16.8" spans="1:8">
       <c r="A19" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
       <c r="D19" s="17"/>
       <c r="E19" s="17"/>
       <c r="F19" s="24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:8">
       <c r="A20" s="17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
       <c r="E20" s="17"/>
       <c r="F20" s="24" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" ht="16.8" spans="1:8">
       <c r="A21" s="25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" s="25"/>
       <c r="C21" s="25"/>
@@ -1969,22 +1970,22 @@
     </row>
     <row r="23" ht="16.8" spans="1:8">
       <c r="A23" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" s="27"/>
       <c r="C23" s="27"/>
       <c r="D23" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E23" s="27"/>
       <c r="F23" s="27"/>
     </row>
-    <row r="24" ht="21" customHeight="1" spans="1:8">
+    <row r="24" ht="34" customHeight="1" spans="1:8">
       <c r="A24" s="28"/>
       <c r="B24" s="29"/>
       <c r="C24" s="30"/>
       <c r="D24" s="28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E24" s="29"/>
       <c r="F24" s="30"/>
@@ -1992,19 +1993,19 @@
     </row>
     <row r="25" ht="16.8" spans="1:8">
       <c r="A25" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="27"/>
       <c r="D25" s="27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E25" s="27"/>
       <c r="F25" s="27"/>
     </row>
     <row r="26" ht="16.8" spans="1:8">
       <c r="A26" s="27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
@@ -2012,9 +2013,9 @@
       <c r="E26" s="27"/>
       <c r="F26" s="27"/>
     </row>
-    <row r="27" ht="66" customHeight="1" spans="1:8">
+    <row r="27" ht="21" customHeight="1" spans="1:8">
       <c r="A27" s="32" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B27" s="32"/>
       <c r="C27" s="32"/>
@@ -2024,7 +2025,7 @@
     </row>
     <row r="28" ht="16.8" spans="1:8">
       <c r="A28" s="33" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B28" s="33"/>
       <c r="C28" s="33"/>
@@ -2034,7 +2035,7 @@
     </row>
     <row r="29" ht="16.8" spans="1:8">
       <c r="A29" s="27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B29" s="27"/>
       <c r="C29" s="27"/>
@@ -2044,7 +2045,7 @@
     </row>
     <row r="30" ht="16.8" spans="1:8">
       <c r="A30" s="27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
@@ -2054,11 +2055,11 @@
     </row>
     <row r="31" ht="16.8" spans="1:8">
       <c r="A31" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B31" s="34"/>
       <c r="C31" s="34" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D31" s="34"/>
       <c r="E31" s="34"/>
@@ -2066,11 +2067,11 @@
     </row>
     <row r="32" ht="16.8" spans="1:8">
       <c r="A32" s="34" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B32" s="34"/>
       <c r="C32" s="34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D32" s="34"/>
       <c r="E32" s="34"/>
@@ -2078,7 +2079,7 @@
     </row>
     <row r="33" ht="16.8" spans="1:6">
       <c r="A33" s="34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B33" s="34"/>
       <c r="C33" s="35"/>
@@ -2088,11 +2089,11 @@
     </row>
     <row r="34" ht="16.8" spans="1:6">
       <c r="A34" s="27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B34" s="27"/>
       <c r="C34" s="27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D34" s="27"/>
       <c r="E34" s="27"/>
@@ -2100,7 +2101,7 @@
     </row>
     <row r="35" ht="16.8" spans="1:6">
       <c r="A35" s="32" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" s="32"/>
       <c r="C35" s="32"/>
@@ -2108,7 +2109,7 @@
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
     </row>
-    <row r="36" ht="16.8" hidden="1" spans="1:6">
+    <row r="36" ht="16.8" spans="1:6">
       <c r="A36" s="6"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
@@ -2117,35 +2118,35 @@
     </row>
     <row r="37" ht="16.8" spans="1:6">
       <c r="A37" s="38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B37" s="38"/>
       <c r="C37" s="38" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D37" s="38"/>
       <c r="E37" s="38"/>
       <c r="F37" s="38"/>
     </row>
-    <row r="38" ht="37.5" customHeight="1" spans="1:6">
+    <row r="38" ht="28" customHeight="1" spans="1:6">
       <c r="A38" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B38" s="39"/>
       <c r="C38" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D38" s="39"/>
       <c r="E38" s="39"/>
       <c r="F38" s="39"/>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:6">
+    <row r="39" ht="23" customHeight="1" spans="1:6">
       <c r="A39" s="40"/>
       <c r="B39" s="40"/>
       <c r="C39" s="38"/>
       <c r="D39" s="38"/>
     </row>
-    <row r="40" ht="30.75" customHeight="1" spans="1:6">
+    <row r="40" ht="20" customHeight="1" spans="1:6">
       <c r="A40" s="41"/>
       <c r="B40" s="41"/>
       <c r="C40" s="38"/>
@@ -2157,7 +2158,7 @@
       <c r="C41" s="38"/>
       <c r="D41" s="38"/>
     </row>
-    <row r="42" ht="47.25" customHeight="1" spans="1:6">
+    <row r="42" ht="21" customHeight="1" spans="1:6">
       <c r="A42" s="41"/>
       <c r="B42" s="41"/>
       <c r="C42" s="38"/>

</xml_diff>